<commit_message>
Actualización automática de bajas: 2026-09-17
</commit_message>
<xml_diff>
--- a/informes/bajas_laliga_2026-09-17.xlsx
+++ b/informes/bajas_laliga_2026-09-17.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,27 +458,81 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sistema (Prueba)</t>
+          <t>Real Madrid</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verificación de carpetas</t>
+          <t>Militão</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Física / Médica</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>El script funciona pero la web requiere revisión de HTML.</t>
+          <t>Rotura Ligamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FC Barcelona</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Gavi</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Física / Médica</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Duda</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Molestias</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Atlético de Madrid</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Koke</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Disciplinaria (Sanción)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cinco Amarillas</t>
         </is>
       </c>
     </row>

</xml_diff>